<commit_message>
Added thesis rmd file, re-organized models, and added models for hse eds and the budget
</commit_message>
<xml_diff>
--- a/data/models/dic_comparison.xlsx
+++ b/data/models/dic_comparison.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,64 +501,80 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2318.67</v>
+        <v>2278.07</v>
       </c>
       <c r="C5" t="n">
-        <v>31.85</v>
+        <v>46.71</v>
       </c>
       <c r="D5" t="n">
-        <v>2350.51</v>
+        <v>2324.78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>v2_pymc</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2318.63</v>
+        <v>2318.67</v>
       </c>
       <c r="C6" t="n">
-        <v>35.68</v>
+        <v>31.85</v>
       </c>
       <c r="D6" t="n">
-        <v>2354.31</v>
+        <v>2350.51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v2_pymc</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2410.37</v>
+        <v>2318.63</v>
       </c>
       <c r="C7" t="n">
-        <v>41.8</v>
+        <v>35.68</v>
       </c>
       <c r="D7" t="n">
-        <v>2452.17</v>
+        <v>2354.31</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2410.37</v>
+      </c>
+      <c r="C8" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2452.17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>2647.42</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C9" t="n">
         <v>25.55</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>2672.97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update minor changes and reruns
</commit_message>
<xml_diff>
--- a/data/models/dic_comparison.xlsx
+++ b/data/models/dic_comparison.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,33 +453,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>v5</t>
+          <t>v7</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2277.96</v>
+        <v>-4174.5</v>
       </c>
       <c r="C2" t="n">
-        <v>46.7</v>
+        <v>46.74</v>
       </c>
       <c r="D2" t="n">
-        <v>2324.66</v>
+        <v>-4127.76</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>v4</t>
+          <t>v6</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2277.99</v>
+        <v>2275.13</v>
       </c>
       <c r="C3" t="n">
-        <v>46.75</v>
+        <v>40.53</v>
       </c>
       <c r="D3" t="n">
-        <v>2324.74</v>
+        <v>2315.66</v>
       </c>
     </row>
     <row r="4">
@@ -492,58 +492,138 @@
         <v>2277.94</v>
       </c>
       <c r="C4" t="n">
-        <v>46.82</v>
+        <v>46.76</v>
       </c>
       <c r="D4" t="n">
-        <v>2324.76</v>
+        <v>2324.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v5</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2318.67</v>
+        <v>2277.99</v>
       </c>
       <c r="C5" t="n">
-        <v>31.85</v>
+        <v>46.78</v>
       </c>
       <c r="D5" t="n">
-        <v>2350.51</v>
+        <v>2324.78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>v6</t>
+          <t>v4</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2394.49</v>
+        <v>2278.04</v>
       </c>
       <c r="C6" t="n">
-        <v>42.13</v>
+        <v>46.75</v>
       </c>
       <c r="D6" t="n">
-        <v>2436.63</v>
+        <v>2324.79</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2318.59</v>
+      </c>
+      <c r="C7" t="n">
+        <v>31.82</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2350.41</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v2a</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2341.27</v>
+      </c>
+      <c r="C8" t="n">
+        <v>28.75</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2370.03</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v2b</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2629.67</v>
+      </c>
+      <c r="C9" t="n">
+        <v>28.66</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2658.33</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>2647.42</v>
-      </c>
-      <c r="C7" t="n">
-        <v>25.55</v>
-      </c>
-      <c r="D7" t="n">
-        <v>2672.97</v>
+      <c r="B10" t="n">
+        <v>2647.45</v>
+      </c>
+      <c r="C10" t="n">
+        <v>25.59</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2673.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v0b</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2665.75</v>
+      </c>
+      <c r="C11" t="n">
+        <v>14.31</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2680.07</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v0a</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2672.02</v>
+      </c>
+      <c r="C12" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2685.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>